<commit_message>
Inclusión de hojas de incompatibilidades y accesibilidades
</commit_message>
<xml_diff>
--- a/docs/source/_static/Datos de prueba.xlsx
+++ b/docs/source/_static/Datos de prueba.xlsx
@@ -5,12 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Salas" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Equipos" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Jueces" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Incomp. jueces" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Incomp. jueces equipos" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Accesibilidad" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="242">
   <si>
     <t xml:space="preserve">Sala</t>
   </si>
@@ -30,7 +33,7 @@
     <t xml:space="preserve">Equipo</t>
   </si>
   <si>
-    <t xml:space="preserve">Club</t>
+    <t xml:space="preserve">Institución</t>
   </si>
   <si>
     <t xml:space="preserve">Correo electrónico</t>
@@ -609,6 +612,9 @@
     <t xml:space="preserve">Juez</t>
   </si>
   <si>
+    <t xml:space="preserve">Intitución(es)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Provincia</t>
   </si>
   <si>
@@ -736,6 +742,15 @@
   </si>
   <si>
     <t xml:space="preserve">Juez UVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incompatibilidad(es)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sala(s) accesible(s)</t>
   </si>
 </sst>
 </file>
@@ -2102,7 +2117,7 @@
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="21.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="16.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="25.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="21.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="14.25"/>
@@ -2120,51 +2135,51 @@
         <v>194</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>2</v>
+        <v>195</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>9</v>
@@ -2173,39 +2188,39 @@
       <c r="D2" s="6"/>
       <c r="E2" s="18"/>
       <c r="F2" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K2" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M2" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O2" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>15</v>
@@ -2214,39 +2229,39 @@
       <c r="D3" s="6"/>
       <c r="E3" s="18"/>
       <c r="F3" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N3" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O3" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>21</v>
@@ -2255,39 +2270,39 @@
       <c r="D4" s="6"/>
       <c r="E4" s="18"/>
       <c r="F4" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N4" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O4" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>27</v>
@@ -2296,39 +2311,39 @@
       <c r="D5" s="6"/>
       <c r="E5" s="18"/>
       <c r="F5" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N5" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>33</v>
@@ -2337,39 +2352,39 @@
       <c r="D6" s="6"/>
       <c r="E6" s="18"/>
       <c r="F6" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N6" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O6" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>39</v>
@@ -2378,39 +2393,39 @@
       <c r="D7" s="6"/>
       <c r="E7" s="18"/>
       <c r="F7" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I7" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M7" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N7" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>45</v>
@@ -2419,39 +2434,39 @@
       <c r="D8" s="6"/>
       <c r="E8" s="18"/>
       <c r="F8" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N8" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>51</v>
@@ -2460,39 +2475,39 @@
       <c r="D9" s="6"/>
       <c r="E9" s="23"/>
       <c r="F9" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M9" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N9" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>57</v>
@@ -2501,39 +2516,39 @@
       <c r="D10" s="6"/>
       <c r="E10" s="18"/>
       <c r="F10" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J10" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L10" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N10" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>63</v>
@@ -2542,39 +2557,39 @@
       <c r="D11" s="6"/>
       <c r="E11" s="18"/>
       <c r="F11" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I11" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M11" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N11" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O11" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>69</v>
@@ -2583,39 +2598,39 @@
       <c r="D12" s="6"/>
       <c r="E12" s="18"/>
       <c r="F12" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I12" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M12" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N12" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O12" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>76</v>
@@ -2624,39 +2639,39 @@
       <c r="D13" s="6"/>
       <c r="E13" s="23"/>
       <c r="F13" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I13" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K13" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L13" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M13" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N13" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O13" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>82</v>
@@ -2665,39 +2680,39 @@
       <c r="D14" s="6"/>
       <c r="E14" s="18"/>
       <c r="F14" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L14" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M14" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N14" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O14" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>88</v>
@@ -2706,39 +2721,39 @@
       <c r="D15" s="6"/>
       <c r="E15" s="18"/>
       <c r="F15" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I15" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J15" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L15" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M15" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N15" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O15" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>94</v>
@@ -2747,39 +2762,39 @@
       <c r="D16" s="6"/>
       <c r="E16" s="18"/>
       <c r="F16" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I16" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N16" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O16" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>101</v>
@@ -2788,39 +2803,39 @@
       <c r="D17" s="6"/>
       <c r="E17" s="23"/>
       <c r="F17" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I17" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L17" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M17" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N17" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O17" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>107</v>
@@ -2829,39 +2844,39 @@
       <c r="D18" s="6"/>
       <c r="E18" s="18"/>
       <c r="F18" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I18" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K18" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N18" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O18" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>113</v>
@@ -2870,39 +2885,39 @@
       <c r="D19" s="6"/>
       <c r="E19" s="18"/>
       <c r="F19" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I19" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K19" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L19" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M19" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N19" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O19" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B20" s="24" t="s">
         <v>188</v>
@@ -2911,39 +2926,39 @@
       <c r="D20" s="6"/>
       <c r="E20" s="18"/>
       <c r="F20" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I20" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L20" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M20" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N20" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O20" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>169</v>
@@ -2952,39 +2967,39 @@
       <c r="D21" s="6"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I21" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J21" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L21" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M21" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N21" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O21" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>119</v>
@@ -2993,39 +3008,39 @@
       <c r="D22" s="6"/>
       <c r="E22" s="18"/>
       <c r="F22" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I22" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K22" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L22" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M22" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N22" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O22" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>126</v>
@@ -3034,39 +3049,39 @@
       <c r="D23" s="6"/>
       <c r="E23" s="23"/>
       <c r="F23" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I23" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L23" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M23" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N23" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O23" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>132</v>
@@ -3075,39 +3090,39 @@
       <c r="D24" s="6"/>
       <c r="E24" s="23"/>
       <c r="F24" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I24" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K24" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L24" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M24" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N24" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O24" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>138</v>
@@ -3116,39 +3131,39 @@
       <c r="D25" s="6"/>
       <c r="E25" s="18"/>
       <c r="F25" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I25" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L25" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M25" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N25" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O25" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B26" s="24" t="s">
         <v>144</v>
@@ -3157,39 +3172,39 @@
       <c r="D26" s="6"/>
       <c r="E26" s="18"/>
       <c r="F26" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I26" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J26" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K26" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L26" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M26" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N26" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O26" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B27" s="24" t="s">
         <v>150</v>
@@ -3198,39 +3213,39 @@
       <c r="D27" s="6"/>
       <c r="E27" s="18"/>
       <c r="F27" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I27" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L27" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M27" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N27" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O27" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B28" s="24" t="s">
         <v>156</v>
@@ -3239,39 +3254,39 @@
       <c r="D28" s="6"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I28" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L28" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M28" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N28" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O28" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B29" s="24" t="s">
         <v>162</v>
@@ -3280,39 +3295,39 @@
       <c r="D29" s="6"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I29" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J29" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M29" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N29" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O29" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B30" s="24" t="s">
         <v>175</v>
@@ -3321,39 +3336,39 @@
       <c r="D30" s="6"/>
       <c r="E30" s="18"/>
       <c r="F30" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I30" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J30" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L30" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M30" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N30" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O30" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>181</v>
@@ -3362,34 +3377,34 @@
       <c r="D31" s="6"/>
       <c r="E31" s="23"/>
       <c r="F31" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I31" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J31" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L31" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M31" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N31" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="O31" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,4 +3574,97 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.3"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>239</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>240</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización instituciones ADUJA y CDUGR
</commit_message>
<xml_diff>
--- a/docs/source/_static/Datos de prueba.xlsx
+++ b/docs/source/_static/Datos de prueba.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Salas" sheetId="1" state="visible" r:id="rId3"/>
@@ -108,6 +108,24 @@
     <t xml:space="preserve">Orador 15</t>
   </si>
   <si>
+    <t xml:space="preserve">ADUJA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 126</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 130</t>
+  </si>
+  <si>
     <t xml:space="preserve">ADUMA</t>
   </si>
   <si>
@@ -216,6 +234,24 @@
     <t xml:space="preserve">Orador 45</t>
   </si>
   <si>
+    <t xml:space="preserve">CDUGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 122</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orador 125</t>
+  </si>
+  <si>
     <t xml:space="preserve">CEU San Pablo</t>
   </si>
   <si>
@@ -495,42 +531,6 @@
     <t xml:space="preserve">Orador 120</t>
   </si>
   <si>
-    <t xml:space="preserve">UGR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 122</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 124</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 125</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UJA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 126</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 127</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 128</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orador 130</t>
-  </si>
-  <si>
     <t xml:space="preserve">UPF</t>
   </si>
   <si>
@@ -663,6 +663,9 @@
     <t xml:space="preserve">Juez ADUEEE</t>
   </si>
   <si>
+    <t xml:space="preserve">Juez ADUJA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juez ADUMA</t>
   </si>
   <si>
@@ -681,6 +684,9 @@
     <t xml:space="preserve">Juez CDU</t>
   </si>
   <si>
+    <t xml:space="preserve">Juez CDUGR</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juez CEU San Pablo</t>
   </si>
   <si>
@@ -730,12 +736,6 @@
   </si>
   <si>
     <t xml:space="preserve">Juez UFV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juez UGR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juez UJA</t>
   </si>
   <si>
     <t xml:space="preserve">Juez URJC</t>
@@ -957,11 +957,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1004,6 +1004,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1014,10 +1018,6 @@
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1042,6 +1042,31 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
     <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0000FF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1450,26 +1475,26 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1546,10 +1571,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
       <c r="C9" s="6"/>
@@ -1570,10 +1595,10 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C10" s="6"/>
@@ -1621,79 +1646,79 @@
       <c r="A12" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="1" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>76</v>
+      <c r="B13" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="G13" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="H13" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="F14" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="G14" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="H14" s="8" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="10" t="s">
         <v>88</v>
       </c>
       <c r="C15" s="6"/>
@@ -1738,58 +1763,58 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>101</v>
+      <c r="B17" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="F17" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="G17" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="H17" s="8" t="s">
         <v>105</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="F18" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="G18" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="H18" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="H18" s="8" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="10" t="s">
         <v>113</v>
       </c>
       <c r="C19" s="6"/>
@@ -1834,58 +1859,58 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>126</v>
+      <c r="B21" s="8" t="s">
+        <v>125</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="F21" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="G21" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="H21" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="H21" s="8" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>132</v>
+      <c r="B22" s="8" t="s">
+        <v>131</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="F22" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="G22" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="H22" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="8" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="10" t="s">
         <v>138</v>
       </c>
       <c r="C23" s="6"/>
@@ -1930,58 +1955,58 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="8" t="s">
         <v>150</v>
       </c>
       <c r="C25" s="6"/>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G25" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="H25" s="8" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="9" t="s">
         <v>156</v>
       </c>
       <c r="C26" s="6"/>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" s="8" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>162</v>
       </c>
       <c r="C27" s="6"/>
@@ -2005,7 +2030,7 @@
       <c r="A28" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="9" t="s">
         <v>169</v>
       </c>
       <c r="C28" s="6"/>
@@ -2026,10 +2051,10 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="9" t="s">
         <v>175</v>
       </c>
       <c r="C29" s="6"/>
@@ -2050,10 +2075,10 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="10" t="s">
         <v>181</v>
       </c>
       <c r="C30" s="6"/>
@@ -2181,7 +2206,7 @@
       <c r="A2" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="17"/>
@@ -2222,7 +2247,7 @@
       <c r="A3" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="17"/>
@@ -2263,7 +2288,7 @@
       <c r="A4" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="17"/>
@@ -2304,7 +2329,7 @@
       <c r="A5" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="17"/>
@@ -2345,7 +2370,7 @@
       <c r="A6" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>33</v>
       </c>
       <c r="C6" s="17"/>
@@ -2386,7 +2411,7 @@
       <c r="A7" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C7" s="17"/>
@@ -2427,7 +2452,7 @@
       <c r="A8" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C8" s="17"/>
@@ -2465,15 +2490,15 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="6"/>
-      <c r="E9" s="23"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="18" t="s">
         <v>209</v>
       </c>
@@ -2506,15 +2531,15 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="17"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="6"/>
-      <c r="E10" s="18"/>
+      <c r="E10" s="24"/>
       <c r="F10" s="18" t="s">
         <v>209</v>
       </c>
@@ -2550,7 +2575,7 @@
       <c r="A11" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>63</v>
       </c>
       <c r="C11" s="17"/>
@@ -2591,7 +2616,7 @@
       <c r="A12" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="21" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="17"/>
@@ -2629,15 +2654,15 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="B13" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="C13" s="22"/>
+      <c r="B13" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="17"/>
       <c r="D13" s="6"/>
-      <c r="E13" s="23"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="18" t="s">
         <v>209</v>
       </c>
@@ -2673,8 +2698,8 @@
       <c r="A14" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>82</v>
+      <c r="B14" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="6"/>
@@ -2711,15 +2736,15 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="C15" s="17"/>
+      <c r="C15" s="23"/>
       <c r="D15" s="6"/>
-      <c r="E15" s="18"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="18" t="s">
         <v>209</v>
       </c>
@@ -2755,7 +2780,7 @@
       <c r="A16" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>94</v>
       </c>
       <c r="C16" s="17"/>
@@ -2793,15 +2818,15 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="B17" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="C17" s="22"/>
+      <c r="B17" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="17"/>
       <c r="D17" s="6"/>
-      <c r="E17" s="23"/>
+      <c r="E17" s="18"/>
       <c r="F17" s="18" t="s">
         <v>209</v>
       </c>
@@ -2837,8 +2862,8 @@
       <c r="A18" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>107</v>
+      <c r="B18" s="10" t="s">
+        <v>106</v>
       </c>
       <c r="C18" s="17"/>
       <c r="D18" s="6"/>
@@ -2875,15 +2900,15 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="C19" s="17"/>
+      <c r="C19" s="23"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="18"/>
+      <c r="E19" s="24"/>
       <c r="F19" s="18" t="s">
         <v>209</v>
       </c>
@@ -2919,8 +2944,8 @@
       <c r="A20" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="B20" s="24" t="s">
-        <v>188</v>
+      <c r="B20" s="10" t="s">
+        <v>119</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="6"/>
@@ -2960,8 +2985,8 @@
       <c r="A21" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>169</v>
+      <c r="B21" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="6"/>
@@ -3001,8 +3026,8 @@
       <c r="A22" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>119</v>
+      <c r="B22" s="21" t="s">
+        <v>188</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="6"/>
@@ -3039,15 +3064,15 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="16" t="s">
         <v>230</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="C23" s="5"/>
+      <c r="B23" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C23" s="17"/>
       <c r="D23" s="6"/>
-      <c r="E23" s="23"/>
+      <c r="E23" s="18"/>
       <c r="F23" s="18" t="s">
         <v>209</v>
       </c>
@@ -3080,15 +3105,15 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="B24" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="22"/>
+      <c r="B24" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" s="17"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="23"/>
+      <c r="E24" s="18"/>
       <c r="F24" s="18" t="s">
         <v>209</v>
       </c>
@@ -3121,15 +3146,15 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="C25" s="17"/>
+      <c r="C25" s="5"/>
       <c r="D25" s="6"/>
-      <c r="E25" s="18"/>
+      <c r="E25" s="24"/>
       <c r="F25" s="18" t="s">
         <v>209</v>
       </c>
@@ -3162,15 +3187,15 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="22" t="s">
         <v>233</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="C26" s="17"/>
+      <c r="C26" s="23"/>
       <c r="D26" s="6"/>
-      <c r="E26" s="18"/>
+      <c r="E26" s="24"/>
       <c r="F26" s="18" t="s">
         <v>209</v>
       </c>
@@ -3206,7 +3231,7 @@
       <c r="A27" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="10" t="s">
         <v>150</v>
       </c>
       <c r="C27" s="17"/>
@@ -3247,7 +3272,7 @@
       <c r="A28" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="21" t="s">
         <v>156</v>
       </c>
       <c r="C28" s="17"/>
@@ -3288,7 +3313,7 @@
       <c r="A29" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="21" t="s">
         <v>162</v>
       </c>
       <c r="C29" s="17"/>
@@ -3329,7 +3354,7 @@
       <c r="A30" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="21" t="s">
         <v>175</v>
       </c>
       <c r="C30" s="17"/>
@@ -3367,15 +3392,15 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="22" t="s">
         <v>238</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="C31" s="22"/>
+      <c r="C31" s="23"/>
       <c r="D31" s="6"/>
-      <c r="E31" s="23"/>
+      <c r="E31" s="24"/>
       <c r="F31" s="18" t="s">
         <v>209</v>
       </c>
@@ -3408,119 +3433,119 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22"/>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="22"/>
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
     </row>
     <row r="34" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22"/>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
+      <c r="A35" s="23"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
     </row>
     <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="22"/>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
     </row>
     <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
+      <c r="A37" s="23"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22"/>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
     </row>
     <row r="41" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="22"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
     </row>
     <row r="42" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="25"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
       <c r="E42" s="26"/>
       <c r="F42" s="26"/>
       <c r="G42" s="27"/>
@@ -3529,8 +3554,8 @@
     </row>
     <row r="43" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="25"/>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
       <c r="E43" s="27"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
@@ -3539,8 +3564,8 @@
     </row>
     <row r="44" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="25"/>
-      <c r="B44" s="22"/>
-      <c r="C44" s="22"/>
+      <c r="B44" s="23"/>
+      <c r="C44" s="23"/>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
@@ -3549,8 +3574,8 @@
     </row>
     <row r="45" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="25"/>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="23"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
@@ -3584,8 +3609,8 @@
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="36.3"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3615,8 +3640,8 @@
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="20.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="36.46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3646,8 +3671,8 @@
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="20.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="36.46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>